<commit_message>
Make XMLTV channel field optional
</commit_message>
<xml_diff>
--- a/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
+++ b/backend/assets/Broadcast_Tool_Pro_XMLTV_Template.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R8127858020a54221"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Redb6dbb3c6c64a7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="Rc154734f7fed4e51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="R9a0bd0b8565d4ee7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programming" sheetId="1" r:id="R9e69d69f6d5f4f78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R4e4e8892d5c24a7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Reference" sheetId="3" r:id="R7c1c86c5fcf24511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="4" r:id="R43173f4e01d44f60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -94,12 +94,12 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFDBEAFE"/>
+        <x:fgColor rgb="FFEEF2F7"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEEF2F7"/>
+        <x:fgColor rgb="FFDBEAFE"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -283,13 +283,13 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -349,13 +349,13 @@
     <xdr:ext cx="419100" cy="390525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="774f9c04-dd49-49d2-974a-9800743969be"/>
+        <xdr:cNvPr id="1" name="321a084d-c9ec-4de5-aedd-12b20f06ca6f"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R3cef7ae509bb48a1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Raf6513508cf1490c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -381,13 +381,13 @@
     <xdr:ext cx="419100" cy="390525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="eeaa3db8-afee-4d57-8d62-f92ed48e1b34"/>
+        <xdr:cNvPr id="1" name="509beddc-86d6-4dc3-9dab-a3d29e55ddd4"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Reeba903cdd804b17"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R91ef6872f57e4bf9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -413,13 +413,13 @@
     <xdr:ext cx="419100" cy="390525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="e89da3f8-2d3e-4602-b710-21843ca2cdba"/>
+        <xdr:cNvPr id="1" name="9e1e2822-3176-4827-97a7-278378adc5f7"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R60666cbcf2544f49"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R195139023c69493e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -445,13 +445,13 @@
     <xdr:ext cx="419100" cy="390525"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="e8e8646d-13fc-4979-bc89-eacdea07f099"/>
+        <xdr:cNvPr id="1" name="42067acf-d435-4122-9756-ec2e74e04350"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7661c9c9247546d9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2da7b0d122d44b4b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -701,12 +701,12 @@
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="15" t="str">
-        <x:v>Channel must match exactly / Channel debe coincidir exactamente · Parental Rating is optional free text / Parental Rating es texto libre opcional.</x:v>
+        <x:v>Channel is optional; blank uses the selected channel / Channel es opcional; vacío usa el canal seleccionado · Parental Rating is optional free text / Parental Rating es texto libre opcional.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="44" customHeight="1">
       <x:c r="A4" s="13" t="str">
-        <x:v>Channel</x:v>
+        <x:v>Channel (Optional)</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
         <x:v>Air Date</x:v>
@@ -14808,7 +14808,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeea4cfcc18a4875"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabb6993fcd764eed"/>
 </x:worksheet>
 </file>
 
@@ -14870,10 +14870,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="41" t="str">
-        <x:v>Channel is required and must exactly match the selected registered channel on every row.</x:v>
+        <x:v>Channel is optional. Leave it blank to use the selected channel, or enter the exact registered name. A mismatch can be replaced through Authorize Suggested Corrections.</x:v>
       </x:c>
       <x:c r="C7" s="41" t="str">
-        <x:v>Channel es obligatorio y debe coincidir exactamente con el canal registrado seleccionado en cada fila.</x:v>
+        <x:v>Channel es opcional. Déjalo vacío para usar el canal seleccionado o ingresa el nombre registrado exacto. Una discrepancia puede reemplazarse mediante Autorizar correcciones sugeridas.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -15059,7 +15059,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3faf98d30e214253"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5239b77cf43e49ee"/>
 </x:worksheet>
 </file>
 
@@ -15104,10 +15104,10 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="62" t="str">
-        <x:v>Channel</x:v>
+        <x:v>Channel (Optional)</x:v>
       </x:c>
       <x:c r="B5" s="62" t="str">
-        <x:v>EN: Exact registered channel name; it must match every row. ES: Nombre exacto del canal registrado; debe coincidir en cada fila.</x:v>
+        <x:v>EN: Leave blank to use the selected channel automatically, or enter its exact registered name. A different name is offered as a suggested correction. ES: Déjalo vacío para usar automáticamente el canal seleccionado o ingresa su nombre registrado exacto. Un nombre diferente se ofrece como corrección sugerida.</x:v>
       </x:c>
       <x:c r="C5" s="62" t="str">
         <x:v>Exact text / Texto exacto</x:v>
@@ -15116,7 +15116,7 @@
         <x:v>Comercio TV</x:v>
       </x:c>
       <x:c r="E5" s="62" t="str">
-        <x:v>Required / Obligatorio</x:v>
+        <x:v>Optional / Opcional</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -15551,7 +15551,7 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d898d4a6079484c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcdcc4113e000405f"/>
 </x:worksheet>
 </file>
 
@@ -15600,7 +15600,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="13" t="str">
-        <x:v>Channel</x:v>
+        <x:v>Channel (Optional)</x:v>
       </x:c>
       <x:c r="B4" s="13" t="str">
         <x:v>Air Date</x:v>
@@ -15839,6 +15839,6 @@
     <x:mergeCell ref="A1:A2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d43e9c13a044b95"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c1beb79d7d54278"/>
 </x:worksheet>
 </file>
</xml_diff>